<commit_message>
Add PO PDF export, procurement settings, and custom PO numbers.
Support downloadable purchase order PDFs with company branding, supplier payment details, currency/tax/discount totals, vendor product name mapping, and optional custom PO numbers on create and edit.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/samples/sample-mappings.xlsx
+++ b/samples/sample-mappings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jessi\Projects\fti-supply-chain\samples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36ECD7CD-DEE6-43B1-9A06-56DE59B2B826}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{007538C5-29F0-48D0-B5B3-5A888F02CECB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14914" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14914" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Franchises" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2654" uniqueCount="601">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2660" uniqueCount="602">
   <si>
     <t>sku_code</t>
   </si>
@@ -1837,6 +1837,9 @@
   </si>
   <si>
     <t>FCR-TMN-ACNESPOTTREATMENT-8ML</t>
+  </si>
+  <si>
+    <t>BND-ILP-LIPBUTTER-MINIS</t>
   </si>
 </sst>
 </file>
@@ -2913,7 +2916,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C1241"/>
+  <dimension ref="A1:C1244"/>
   <sheetFormatPr defaultRowHeight="15.9" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="45.85546875" bestFit="1" customWidth="1"/>
@@ -16568,6 +16571,39 @@
         <v>12</v>
       </c>
       <c r="C1241">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1242" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1242" t="s">
+        <v>601</v>
+      </c>
+      <c r="B1242" t="s">
+        <v>103</v>
+      </c>
+      <c r="C1242">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1243" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1243" t="s">
+        <v>601</v>
+      </c>
+      <c r="B1243" t="s">
+        <v>104</v>
+      </c>
+      <c r="C1243">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1244" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1244" t="s">
+        <v>601</v>
+      </c>
+      <c r="B1244" t="s">
+        <v>105</v>
+      </c>
+      <c r="C1244">
         <v>1</v>
       </c>
     </row>

</xml_diff>